<commit_message>
Route X reproduces on the merged data; "If you miss a leg" rebuilt for the booked chain
231.87 h against the sheet's 232.30 (router's shorter Fargo finish). Without
Jefferson 21:15 Chicago -> Omaha and 06:15 Omaha -> Sioux Falls it is 256.37 h.
scripts/x_miss.py (leaf script, nothing imports it, so regress.py not rerun)
costs a miss at every booked ride against catching it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_itinerary_nov12.xlsx
+++ b/docs/x_itinerary_nov12.xlsx
@@ -3416,1331 +3416,1298 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>STALE: computed for the Oct 15 chain (SLC airport walk, Houston METRORail, morning Kenosha). Recompute once the Four Winds / Jefferson / Moorhead trips are in the repo.</t>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>missed</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>next best</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cost h</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>recovery starts with</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>missed</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>from</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>to</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>next best finish</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>cost h</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>recovery starts with</t>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>d1 Thu 22:20 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>d2 Fri 22:20 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Billings</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d1 Thu 22:20 Jefferson Lines</t>
+          <t>d2 Fri 01:30 Jefferson Lines</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson)</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>24</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>d2 Fri 22:20 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Billings</t>
+          <t>d2 Fri 11:30 Jefferson Lines: Billings -&gt; Whitefish</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>d2 Fri 01:30 Jefferson Lines</t>
+          <t>d2 Fri 10:45 Northwestern Stage Lines</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>168</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>d2 Fri 11:30 Jefferson Lines: Billings -&gt; Whitefish</t>
+          <t>d2 Fri 11:10 FlixBus-us: Spokane Station -&gt; Pasco Bus Stop</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>d2 Fri 10:45 Northwestern Stage Lines</t>
+          <t>d2 Fri 13:25 Greyhound-us</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Provo Intermodal Hub</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>24</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>d2 Fri 11:10 FlixBus-us: Spokane Station -&gt; Pasco Bus Stop</t>
+          <t>d2 Fri 14:40 FlixBus-us: Pasco Bus Stop -&gt; Portland Curbside Bus Stop</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>d2 Fri 13:25 Greyhound-us</t>
+          <t>d3 Sat 07:45 Salt Lake Express</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Provo Central Station/Intermodal Hub</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Salt Lake City Intermodal Trans Ctr</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>24</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>d2 Fri 14:40 FlixBus-us: Pasco Bus Stop -&gt; Portland Curbside Bus Stop</t>
+          <t>d3 Sat 08:40 Salt Lake Express: Provo/Orem (Exit 263) -&gt; Salt Lake City (Shop)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>d3 Sat 04:45 Salt Lake Express</t>
+          <t>d3 Sat 12:40 Salt Lake Express</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>24</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>d3 Sat 06:00 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
+          <t>d3 Sat 13:45 Salt Lake Express: Saint George (Shop) -&gt; Las Vegas (Airport)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>d3 Sat 10:30 Salt Lake Express</t>
+          <t>d3 Sat 15:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>Las Vegas Strip (Las Vegas Blvd)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>Barstow Station</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>24</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>d3 Sat 12:15 Salt Lake Express: Saint George (Shop) -&gt; Las Vegas (Airport)</t>
+          <t>d3 Sat 18:45 Greyhound-us: Las Vegas Bus Terminal -&gt; Los Angeles Union Station</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>d3 Sat 14:00 Greyhound-us</t>
+          <t>d3 Sat 20:47 Amtrak</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Barstow (Amtrak)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>168</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>24</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>d3 Sat 15:15 702 Shuttles: Las Vegas Dean Martin Blue Diamond (702 Shuttles) -&gt; Fontana 3892 Sierra Ave ampm (702 Shuttles)</t>
+          <t>d3 Sat 22:25 FlixBus-us: Barstow Station -&gt; Las Vegas Strip (Las Vegas Blvd)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>d3 Sat 18:43 Amtrak</t>
+          <t>d5 Mon 03:00 BeeLine Express-Village Travel</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>d18 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>168</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>d3 Sat 18:55 Greyhound-us: San Bernardino Depot -&gt; Las Vegas Bus Terminal</t>
+          <t>d5 Mon 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>d5 Mon 03:00 BeeLine Express-Village Travel</t>
+          <t>d5 Mon 08:35 FlixBus-us</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>d15 Thu 15:28</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>96</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>24</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>d5 Mon 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+          <t>d5 Mon 14:05 Greyhound-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>d5 Mon 06:55 Greyhound-us</t>
+          <t>d5 Mon 13:00 Greyhound-us</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
+          <t>Houston Bus Station (Greyhound)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>d15 Thu 15:28</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>96</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>24</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>d5 Mon 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Downtown Houston (Gray St.)</t>
+          <t>d5 Mon 15:00 Vonlane (premium coach): Dallas DoubleTree Love Field (Vonlane) -&gt; Houston Hyatt Regency Downtown (Vonlane)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>d5 Mon 11:30 FlixBus-us</t>
+          <t>d5 Mon 18:35 Greyhound-us</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
+          <t>Houston Bus Station (Greyhound)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Downtown Houston (Gray St.)</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>d15 Thu 15:28</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>96</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>24</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>d5 Mon 11:45 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
+          <t>d5 Mon 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>d5 Mon 16:50 Metropolitan Transit Authority of Harris County</t>
+          <t>d6 Tue 11:25 Greyhound-us</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Central Station Rusk EB</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Magnolia Park Transit Center EB</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>d15 Thu 15:28</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>96</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>24</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>d5 Mon 17:02 Metropolitan Transit Authority of Harris County: Central Station Rusk EB -&gt; Magnolia Park Transit Center EB</t>
+          <t>d6 Tue 12:50 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Atlanta Bus Station</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>d5 Mon 18:35 Greyhound-us</t>
+          <t>d6 Tue 15:00 Jacksonville Transportation Authority</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Houston Bus Station (Greyhound)</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Amtrak Station</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>d15 Thu 15:28</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>96</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>d5 Mon 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
+          <t>d6 Tue 16:11 Amtrak: Jacksonville -&gt; Washington Union Station</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d6 Tue 11:25 Greyhound-us</t>
+          <t>d6 Tue 16:11 Amtrak</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>d14 Wed 15:28</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>72</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>24</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>d6 Tue 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
+          <t>d6 Tue 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d6 Tue 15:00 Jacksonville Transportation Authority</t>
+          <t>d7 Wed 06:50 Amtrak</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>24</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>d6 Tue 15:30 Jacksonville Transportation Authority: JRTC Bay H -&gt; Amtrak Station</t>
+          <t>d7 Wed 07:06 Amtrak: Washington Union Station -&gt; Philadelphia</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d6 Tue 16:11 Amtrak</t>
+          <t>d7 Wed 14:30 Dartmouth Coach</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>24</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>d6 Tue 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
+          <t>d7 Wed 15:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d7 Wed 06:45 Amtrak</t>
+          <t>d7 Wed 17:10 Advance Transit</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Sykes Ave @ Greyhound</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>d14 Wed 15:28</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>72</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>24</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>d7 Wed 07:06 Amtrak: Washington Union Station -&gt; Stamford Amtrak Station</t>
+          <t>d7 Wed 17:23 Advance Transit: Hanover Inn -&gt; Vail DMS</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d7 Wed 14:30 Dartmouth Coach</t>
+          <t>d7 Wed 17:55 Greyhound-us</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Boston (South Station)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>24</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>d7 Wed 15:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
+          <t>d7 Wed 22:25 FlixBus-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d7 Wed 17:10 Advance Transit</t>
+          <t>d7 Wed 20:25 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sykes Ave @ Greyhound</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>d7 Wed 17:23 Advance Transit: Hanover Inn -&gt; Vail DMS</t>
+          <t>d7 Wed 20:40 Plymouth &amp; Brockton Street Railway Co.: South Station Transp. Ctr -&gt; Logan International Airport</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d7 Wed 17:55 Greyhound-us</t>
+          <t>d8 Thu 03:15 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>d7 Wed 22:25 FlixBus-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
+          <t>d8 Thu 04:15 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d7 Wed 20:25 Concord Coach Lines</t>
+          <t>d8 Thu 06:10 Amtrak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Ny Moynihan Train Hall At Penn Station</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>d7 Wed 20:40 Plymouth &amp; Brockton Street Railway Co.: South Station Transp. Ctr -&gt; Logan International Airport</t>
+          <t>d8 Thu 07:00 Amtrak: Boston -&gt; Philadelphia</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d8 Thu 03:15 Concord Coach Lines</t>
+          <t>d8 Thu 10:52 Amtrak</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Ny Moynihan Train Hall At Penn Station</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Harrisburg</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>d8 Thu 04:15 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+          <t>d8 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Philadelphia</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d8 Thu 06:10 Amtrak</t>
+          <t>d8 Thu 14:50 Greyhound-us</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Harrisburg Bus Station</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Ny Moynihan Train Hall At Penn Station</t>
+          <t>Indianapolis Bus Station</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>24</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>d8 Thu 07:00 Amtrak: Boston -&gt; Philadelphia</t>
+          <t>d8 Thu 15:03 Amtrak: Harrisburg -&gt; Philadelphia</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
+        <v>30</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>d9 Fri 04:40 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Nashville Bus Station</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
         <v>24</v>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>d8 Thu 10:52 Amtrak</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Ny Moynihan Train Hall At Penn Station</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Harrisburg</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>24</v>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>d8 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Philadelphia</t>
+          <t>d9 Fri 05:20 Greyhound-us: Indianapolis Bus Station -&gt; Lafayette Bus Stop</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d8 Thu 14:50 Greyhound-us</t>
+          <t>d9 Fri 11:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Harrisburg Bus Station</t>
+          <t>Nashville Bus Station</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
         <v>24</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>d8 Thu 19:50 Greyhound-us: Harrisburg Bus Station -&gt; Indianapolis Bus Station</t>
+          <t>d9 Fri 17:00 Greyhound-us: Nashville Bus Station -&gt; Memphis Bus Station</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d9 Fri 04:40 Greyhound-us</t>
+          <t>d9 Fri 15:14 MATA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>AIRWAYS TRANSIT CENTER</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nashville Bus Station</t>
+          <t>NORRIS ROAD at ELVIS PRESLEY BOULEVARD</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>24</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>d9 Fri 05:20 Greyhound-us: Indianapolis Bus Station -&gt; Lafayette Bus Stop</t>
+          <t>d9 Fri 16:00 MATA: AIRWAYS TRANSIT CENTER -&gt; AIRWAYS BOULEVARD at HOLMES ROAD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d9 Fri 11:30 FlixBus-us</t>
+          <t>d9 Fri 15:45 MATA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Nashville Bus Station</t>
+          <t>ELVIS PRESLEY BOULEVARD at EFFIE ROAD</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>HOLMES at ELVIS PRESLEY</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
         <v>24</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>d9 Fri 17:00 Greyhound-us: Nashville Bus Station -&gt; Memphis Bus Station</t>
+          <t>d9 Fri 16:09 MATA: PERRY ROAD at DUNN AVENUE -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d9 Fri 15:14 MATA</t>
+          <t>d9 Fri 17:07 MATA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>HOLMES at ELVIS PRESLEY</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>AIRWAYS TRANSIT CENTER</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>NORRIS ROAD at ELVIS PRESLEY BOULEVARD</t>
-        </is>
-      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
         <v>24</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>d9 Fri 15:45 MATA: AIRWAYS TRANSIT CENTER -&gt; ELLISTON ROAD at CORRY ROAD</t>
+          <t>d9 Fri 17:28 MATA: HOLMES ROAD at CRESSER STREET -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d9 Fri 15:45 MATA</t>
+          <t>d9 Fri 17:45 Greyhound-us</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ELVIS PRESLEY BOULEVARD at EFFIE ROAD</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>HOLMES at ELVIS PRESLEY</t>
+          <t>St Louis Bus Station</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
         <v>24</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>d9 Fri 16:09 MATA: PERRY ROAD at DUNN AVENUE -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
+          <t>d9 Fri 18:14 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d9 Fri 17:07 MATA</t>
+          <t>d9 Fri 23:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HOLMES at ELVIS PRESLEY</t>
+          <t>St Louis Bus Station</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AIRWAYS TRANSIT CENTER</t>
+          <t>Chicago (95th - Dan Ryan)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>d9 Fri 17:28 MATA: HOLMES ROAD at CRESSER STREET -&gt; ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
+          <t>d10 Sat 04:30 Amtrak: St. Louis -&gt; Chicago Union Station</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d9 Fri 17:45 Greyhound-us</t>
+          <t>d10 Sat 06:32 Metra</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>Chicago OTC</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>St Louis Bus Station</t>
+          <t>Kenosha</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>d9 Fri 18:14 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
+          <t>d10 Sat 08:25 Amtrak: Chicago Union Station -&gt; Milwaukee</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>d9 Fri 23:30 FlixBus-us</t>
+          <t>d10 Sat 09:08 Metra</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>St Louis Bus Station</t>
+          <t>Kenosha</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>Chicago OTC</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>d10 Sat 04:30 Amtrak: St. Louis -&gt; Chicago Union Station</t>
+          <t>d10 Sat 09:30 Wisconsin Coach Lines: Metro Train Station - 13th Avenue and 54th Street -&gt; Mitchell Airport</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d10 Sat 06:32 Metra</t>
+          <t>d10 Sat 11:50 Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Chicago OTC</t>
+          <t>35th &amp; State St (Four Winds shuttle)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kenosha</t>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>24</v>
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>d10 Sat 08:32 Metra: Chicago OTC -&gt; Kenosha</t>
+          <t>d10 Sat 13:50 Four Winds Casino Shuttle (Chinatown): 35th &amp; State St (Four Winds shuttle) -&gt; Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d10 Sat 09:08 Metra</t>
+          <t>d10 Sat 18:30 ET Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kenosha</t>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Chicago OTC</t>
+          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>d11 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="n">
+          <t>no loss</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>d10 Sat 09:30 Wisconsin Coach Lines: Metro Train Station - 13th Avenue and 54th Street -&gt; Mitchell Airport</t>
+          <t>d10 Sat 19:00 Four Winds Casino Shuttle (Chinatown): Four Winds Casino New Buffalo MI (shuttle) -&gt; 2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>d10 Sat 11:50 Four Winds Casino Shuttle (Chinatown)</t>
+          <t>d10 Sat 21:15 Jefferson Lines</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>35th &amp; State St (Four Winds shuttle)</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>d11 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="n">
-        <v>0</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>24</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>d10 Sat 13:50 Four Winds Casino Shuttle (Chinatown): 35th &amp; State St (Four Winds shuttle) -&gt; Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>d10 Sat 22:50 Greyhound-us: Chicago Bus Station -&gt; Indianapolis Bus Station</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>d10 Sat 15:00 Four Winds Casino Shuttle (Chinatown)</t>
+          <t>d11 Sun 06:15 Jefferson Lines</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>d11 Sun 15:28</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="n">
-        <v>0</v>
+          <t>+24 h</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>24</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>d10 Sat 17:00 Four Winds Casino Shuttle (Chinatown): Four Winds Casino New Buffalo MI (shuttle) -&gt; 2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+          <t>d12 Mon 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>d10 Sat 21:15 Jefferson Lines</t>
+          <t>d11 Sun 10:00 Jefferson Lines</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>24</v>
+          <t>+8 h</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>8</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>d10 Sat 22:50 Greyhound-us: Chicago Bus Station -&gt; Indianapolis Bus Station</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>d11 Sun 06:15 Jefferson Lines</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Omaha</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Sioux Falls</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>d12 Mon 15:28</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>d12 Mon 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+          <t>d11 Sun 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
-        <v>39</v>
-      </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>d11 Sun 10:00 Jefferson Lines</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Sioux Falls</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Fargo</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>d12 Mon 00:53</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>d11 Sun 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+          <t>Recovery keeps the remaining states in route X's order, from the missed ride's boarding stop one minute after it leaves; cost is against catching it. Built on the repo data as of Oct 5 2026 (timetable window from Sep 24).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
x_miss: X's booked dates (Thu Nov 12, November router; the migration had put it on Nov 5, before Acela 2152 returns), refresh the miss-a-leg sheet
Leaf script, regress not rerun.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_itinerary_nov12.xlsx
+++ b/docs/x_itinerary_nov12.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X itinerary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start day" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="If you miss a leg" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verify" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Book ahead" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="X itinerary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Start day" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="If you miss a leg" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Verify" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Book ahead" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3471,15 +3471,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>d2 Fri 22:20 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Billings</t>
+          <t>d2 Fri 06:35 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Vivian</t>
         </is>
       </c>
     </row>
@@ -3504,11 +3504,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3570,11 +3570,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3603,11 +3603,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3636,11 +3636,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3669,11 +3669,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3702,11 +3702,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>+32 h</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3768,15 +3768,15 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>d5 Mon 14:05 Greyhound-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
+          <t>d5 Mon 10:15 Vonlane: Oklahoma City Omni (Vonlane) -&gt; Dallas DoubleTree Love Field (Vonlane)</t>
         </is>
       </c>
     </row>
@@ -3801,11 +3801,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -3834,11 +3834,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3867,11 +3867,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3933,11 +3933,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>+24 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>d7 Wed 07:06 Amtrak: Washington Union Station -&gt; Philadelphia</t>
+          <t>d7 Wed 07:10 Amtrak: Washington Union Station -&gt; Philadelphia</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>d8 Thu 07:00 Amtrak: Boston -&gt; Philadelphia</t>
+          <t>d8 Thu 07:00 Amtrak: Boston -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>d8 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Philadelphia</t>
+          <t>d8 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>d9 Fri 17:00 Greyhound-us: Nashville Bus Station -&gt; Memphis Bus Station</t>
+          <t>d9 Fri 14:00 Vonlane: Nashville Omni Downtown (Vonlane) -&gt; Memphis Hilton, Ridge Lake Blvd (Vonlane)</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>d9 Fri 16:09 MATA: PERRY ROAD at DUNN AVENUE -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
+          <t>d9 Fri 16:07 MATA: PERRY ROAD at DUNN AVENUE -&gt; SOUTH PARKWAY EAST at BELLEVUE BOULEVARD</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>d9 Fri 17:28 MATA: HOLMES ROAD at CRESSER STREET -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
+          <t>d9 Fri 17:26 MATA: HOLMES ROAD at WALDRUP STREET -&gt; ELVIS PRESLEY BLVD at SOUTH PARKWAY EAST</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>d9 Fri 18:14 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
+          <t>d9 Fri 18:12 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>d10 Sat 04:30 Amtrak: St. Louis -&gt; Chicago Union Station</t>
+          <t>d9 Fri 23:45 FlixBus-us: St Louis Bus Station -&gt; Carbondale Intermodal Station</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>d10 Sat 08:25 Amtrak: Chicago Union Station -&gt; Milwaukee</t>
+          <t>d10 Sat 08:25 Amtrak: Chicago Union Station -&gt; Sturtevant Amtrak Station</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>d10 Sat 22:50 Greyhound-us: Chicago Bus Station -&gt; Indianapolis Bus Station</t>
+          <t>d11 Sun 06:30 Greyhound-us: Davenport (Ground Transportation) -&gt; Chicago Bus Station</t>
         </is>
       </c>
     </row>
@@ -4707,7 +4707,7 @@
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>Recovery keeps the remaining states in route X's order, from the missed ride's boarding stop one minute after it leaves; cost is against catching it. Built on the repo data as of Oct 5 2026 (timetable window from Sep 24).</t>
+          <t>Recovery keeps the remaining states in route X's order, from the missed ride's boarding stop one minute after it leaves; cost is against catching it. Built on the repo data as of Oct 13 2026 (November timetables, X from Thu Nov 12).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NWL Pasco 15:00 -> Oregon -> Boise (t461) and SLE Boise 21:15 -> Pocatello (t462), from Nick's screenshots: the Pasco backup
Missing X's Greyhound 13:25 at Pasco now costs nothing (was +32 h): NWL to Boise, SLE to Pocatello, then the feed's
Pocatello 03:40 -> SLC Airport 06:45 -> Saint George 12:20. Miss-a-leg sheet refreshed. regress.py 15/15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_itinerary_nov12.xlsx
+++ b/docs/x_itinerary_nov12.xlsx
@@ -3570,15 +3570,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+32 h</t>
+          <t>no loss</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>d2 Fri 14:40 FlixBus-us: Pasco Bus Stop -&gt; Portland Curbside Bus Stop</t>
+          <t>d2 Fri 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Boise (Airport)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ride kit: hand-checked backups (Pasco NWL chain, the 702 Shuttles + run as last ditch, the Phoenix Greyhound after a missed Chief) on the miss-a-leg sheet; x_miss writes them every run
Leaf script, regress not rerun.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_itinerary_nov12.xlsx
+++ b/docs/x_itinerary_nov12.xlsx
@@ -3401,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4708,6 +4708,27 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Recovery keeps the remaining states in route X's order, from the missed ride's boarding stop one minute after it leaves; cost is against catching it. Built on the repo data as of Oct 13 2026 (November timetables, X from Thu Nov 12).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pasco, missed Greyhound 13:25: Northwestern 15:00 -&gt; Hermiston -&gt; Pendleton -&gt; La Grande -&gt; Boise 21:10, Salt Lake Express 21:15 -&gt; Pocatello 01:05, 03:40 -&gt; SLC Airport 06:40, 06:45 -&gt; Saint George 12:20. Same Saint George arrival as X: no loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Las Vegas, missed Flix 15:30 (LAST DITCH, not a plan): RTC Red line + 217 from the airport to Blue Diamond, 702 Shuttles 18:15 -&gt; Barstow (1611 E Main) 20:27, then RUN 2.5 mi to Barstow Amtrak for the Chief at 20:47. Needs ~8 mph and an on-time shuttle; the router misses it by one minute even at 9.4 mph with a 5 min boarding allowance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Southwest Chief, missed at Barstow: Greyhound Los Angeles 23:30 -&gt; Phoenix -&gt; Tucson -&gt; Lordsburg NM -&gt; El Paso -&gt; Dallas 06:35 two days on gets AZ NM TX back to Dallas before the 13:00 to Houston in X, but skips CO KS OK. Cost: see docs/sweep.md (Chief miss).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ride kit: the 702 Shuttles + 2.5 mi run is a fit-run backup (platform 20:43, Chief 20:47; the router's 5 min boarding allowance double-counts a run that ends on the platform)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_itinerary_nov12.xlsx
+++ b/docs/x_itinerary_nov12.xlsx
@@ -4704,6 +4704,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
@@ -4711,6 +4712,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
@@ -4721,7 +4723,7 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>Las Vegas, missed Flix 15:30 (LAST DITCH, not a plan): RTC Red line + 217 from the airport to Blue Diamond, 702 Shuttles 18:15 -&gt; Barstow (1611 E Main) 20:27, then RUN 2.5 mi to Barstow Amtrak for the Chief at 20:47. Needs ~8 mph and an on-time shuttle; the router misses it by one minute even at 9.4 mph with a 5 min boarding allowance.</t>
+          <t>Las Vegas, missed Flix 15:30 (FIT-RUN BACKUP): RTC Red line + 217 from the airport to Blue Diamond, 702 Shuttles 18:15 -&gt; Barstow (1611 E Main) 20:27, then RUN 2.5 mi to the Barstow Amtrak platform: at 9.4 mph on the platform 20:43, 4 min before the Chief leaves at 20:47 (and it often runs late). The router shows it missed by a minute only because it adds a 5 min boarding allowance to every connection, which double-counts a run that ends on the platform.</t>
         </is>
       </c>
     </row>

</xml_diff>